<commit_message>
Add time-varying capacity bounds and carbon market
- Make technology_upper_bound, technology_lower_bound,
  new_technology_upper_bound, new_technology_lower_bound
  indexed by (zone, tech, year) instead of (tech, zone)
- Re-introduce technology_lower_bound constraint on cap_existing
- Add carbon market: carbon_offset variable, carbon_tax cost,
  carbon_offset_price cost, fractional carbon_offset_limit
  (offset <= rate * raw zonal emissions)
- carbon_capacity now nets out purchased offsets
- Migrate input Excel files to new shapes; defaults preserve
  prior behavior (lower bounds = 0, tax = 0, offset rate = 0)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/new_technology_upper_bound.xlsx
+++ b/input/new_technology_upper_bound.xlsx
@@ -1,43 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/energy/Documents/research/prep-shot-data/PREP-SHOT/input/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59F838F-A15C-BE4D-BED8-32F4C0120C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="12">
+  <si>
+    <t>zone</t>
+  </si>
   <si>
     <t>tech</t>
   </si>
   <si>
+    <t>BA1</t>
+  </si>
+  <si>
+    <t>BA2</t>
+  </si>
+  <si>
+    <t>BA3</t>
+  </si>
+  <si>
     <t>Coal</t>
   </si>
   <si>
@@ -53,26 +46,17 @@
     <t>Storage</t>
   </si>
   <si>
-    <t>zone</t>
+    <t>year</t>
   </si>
   <si>
     <t>inf</t>
-  </si>
-  <si>
-    <t>BA1</t>
-  </si>
-  <si>
-    <t>BA2</t>
-  </si>
-  <si>
-    <t>BA3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,8 +67,10 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -95,12 +81,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -109,7 +110,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -118,14 +119,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -413,96 +406,647 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="J2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="O2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5" s="1">
+        <v>2020</v>
+      </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>7</v>
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" t="s">
+        <v>11</v>
+      </c>
+      <c r="K5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O5" t="s">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" s="1">
+        <v>2021</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" t="s">
+        <v>11</v>
+      </c>
+      <c r="K6" t="s">
+        <v>11</v>
+      </c>
+      <c r="L6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6" t="s">
+        <v>11</v>
+      </c>
+      <c r="O6" t="s">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" s="1">
+        <v>2022</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K7" t="s">
+        <v>11</v>
+      </c>
+      <c r="L7" t="s">
+        <v>11</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="s">
+        <v>11</v>
+      </c>
+      <c r="O7" t="s">
+        <v>11</v>
+      </c>
+      <c r="P7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="A8" s="1">
+        <v>2023</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" t="s">
+        <v>11</v>
+      </c>
+      <c r="L8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" t="s">
+        <v>11</v>
+      </c>
+      <c r="O8" t="s">
+        <v>11</v>
+      </c>
+      <c r="P8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="A9" s="1">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" t="s">
+        <v>11</v>
+      </c>
+      <c r="K9" t="s">
+        <v>11</v>
+      </c>
+      <c r="L9" t="s">
+        <v>11</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="s">
+        <v>11</v>
+      </c>
+      <c r="O9" t="s">
+        <v>11</v>
+      </c>
+      <c r="P9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="A10" s="1">
+        <v>2025</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10" t="s">
+        <v>11</v>
+      </c>
+      <c r="L10" t="s">
+        <v>11</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10" t="s">
+        <v>11</v>
+      </c>
+      <c r="O10" t="s">
+        <v>11</v>
+      </c>
+      <c r="P10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="A11" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K11" t="s">
+        <v>11</v>
+      </c>
+      <c r="L11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11" t="s">
+        <v>11</v>
+      </c>
+      <c r="O11" t="s">
+        <v>11</v>
+      </c>
+      <c r="P11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12" s="1">
+        <v>2027</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" t="s">
+        <v>11</v>
+      </c>
+      <c r="K12" t="s">
+        <v>11</v>
+      </c>
+      <c r="L12" t="s">
+        <v>11</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12" t="s">
+        <v>11</v>
+      </c>
+      <c r="O12" t="s">
+        <v>11</v>
+      </c>
+      <c r="P12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" s="1">
+        <v>2028</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" t="s">
+        <v>11</v>
+      </c>
+      <c r="K13" t="s">
+        <v>11</v>
+      </c>
+      <c r="L13" t="s">
+        <v>11</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13" t="s">
+        <v>11</v>
+      </c>
+      <c r="O13" t="s">
+        <v>11</v>
+      </c>
+      <c r="P13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="A14" s="1">
+        <v>2029</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="s">
+        <v>11</v>
+      </c>
+      <c r="J14" t="s">
+        <v>11</v>
+      </c>
+      <c r="K14" t="s">
+        <v>11</v>
+      </c>
+      <c r="L14" t="s">
+        <v>11</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14" t="s">
+        <v>11</v>
+      </c>
+      <c r="O14" t="s">
+        <v>11</v>
+      </c>
+      <c r="P14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="A15" s="1">
+        <v>2030</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" t="s">
+        <v>11</v>
+      </c>
+      <c r="L15" t="s">
+        <v>11</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15" t="s">
+        <v>11</v>
+      </c>
+      <c r="O15" t="s">
+        <v>11</v>
+      </c>
+      <c r="P15" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <mergeCells count="3">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="L1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>